<commit_message>
updated chapter45-5 and add objective docs
</commit_message>
<xml_diff>
--- a/data/Quarto_YAMLs.xlsx
+++ b/data/Quarto_YAMLs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R入門\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB83441D-0C44-45C1-AE7B-C77890CD7BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C7D3D5-7F5F-4503-B417-857B222B555B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="6" xr2:uid="{BD8A1D6D-0391-4D96-8986-F577B78F0501}"/>
   </bookViews>

</xml_diff>

<commit_message>
ver.0.4.4.7.1 Shiny apps in the documents were updated
</commit_message>
<xml_diff>
--- a/data/Quarto_YAMLs.xlsx
+++ b/data/Quarto_YAMLs.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R入門\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A749EB1A-C386-4946-AE8B-B8731214CE64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB3F771-3A99-49C8-A560-2A23D712C947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19230" yWindow="2880" windowWidth="20775" windowHeight="11835" activeTab="7" xr2:uid="{BD8A1D6D-0391-4D96-8986-F577B78F0501}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="16440" activeTab="7" xr2:uid="{BD8A1D6D-0391-4D96-8986-F577B78F0501}"/>
   </bookViews>
   <sheets>
     <sheet name="format" sheetId="1" r:id="rId1"/>
@@ -1753,6 +1748,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1816,6 +1812,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2030,6 +2027,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2112,6 +2110,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2271,6 +2270,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2441,6 +2441,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2576,6 +2577,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2702,5 +2704,6 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>